<commit_message>
Release v0.10.0: NAAC 2.6.1 evidence pack
An editable Word document per programme for NAAC's university-manual
metric 2.6.1 (learning outcomes stated, integrated into assessment, made
public, and their attainment evaluated), assembled from what the tool
already knows.

- evidence.py (python-docx, now a dependency): A4; Before submission
  (what the data shows still needs doing), programme outcomes or the
  framework used, every course's outcomes with Bloom levels, the CO-PO
  articulation matrix (landscape page, shaded by strength), attainment
  for a batch, an actions table for outcomes below target, and the method
- `curintel evidence PROGRAMME [--attainment RESULTS]`
- API: POST /api/programmes/{id}/evidence.docx, with or without a
  batch's results; web app: a download button in the attainment panel
- Framework.own marks a programme's own outcomes
- Sample evidence pack (fictional) in docs/

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/programme-template.xlsx
+++ b/docs/programme-template.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Programme" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Courses" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Credit scheme" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Programme outcomes" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="How to fill" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Programme" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Courses" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Credit scheme" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Programme outcomes" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How to fill" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>